<commit_message>
S32: Beam saw 20/10 corrected end time (18:15-18:18)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HsFNnGJRzg6EEfnut1VvMX
</commit_message>
<xml_diff>
--- a/loss-time/outputs/Loss_time_S32_05-10_den_20-10.xlsx
+++ b/loss-time/outputs/Loss_time_S32_05-10_den_20-10.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="875" uniqueCount="199">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="875" uniqueCount="198">
   <si>
     <t xml:space="preserve">LOSS TIME MÃ S32 (OTHER SUPPORT OF PRODUCTION) - 05/10 ĐẾN 20/10/2026 - LÀM RIÊNG, KHÔNG LẪN MÃ KHÁC</t>
   </si>
@@ -344,9 +344,6 @@
     <t xml:space="preserve">CZ567F09</t>
   </si>
   <si>
-    <t xml:space="preserve">Charge to: Unassigned; Nguồn ghi 18:15-18:13 (giờ kết thúc nhỏ hơn giờ bắt đầu, -0.1 giờ)</t>
-  </si>
-  <si>
     <t xml:space="preserve">code 191</t>
   </si>
   <si>
@@ -599,10 +596,10 @@
     <t xml:space="preserve">1. Bảng này CHỈ chứa mã S32, tách hoàn toàn khỏi bảng P20/P26/P22/A2 (không lẫn mã khác). Khi bạn cập nhật, tôi giữ nguyên nguyên tắc này.</t>
   </si>
   <si>
-    <t xml:space="preserve">2. Nguồn: 5 file trong gói zip (lấy bản mới nhất mỗi loại: Beam saw bản 20/10, UV bản (1), Ép nóng bản (1), Veneer bản 20/10) và 3 hình (thợ sơn tuần 42, cào cước 16/10, bắn cát 15/10). Chỉ lấy dòng từ 05/10 đến 20/10. UV (báo cáo ngày đến 11/10, phát sinh đến 13/10) và Ép nóng (đến 6/10) chưa có số liệu mới.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3. Tất cả giờ công trong bảng khớp với số giờ trong nguồn (sheet "Đối chiếu nguồn"). Tổng giờ công xem sheet "Đối chiếu nguồn". Riêng dòng Beam saw 20/10 (18:15-18:13) nguồn ghi -0,1 giờ nên bảng ghi 0 giờ và không tính vào đối chiếu.</t>
+    <t xml:space="preserve">2. Nguồn: 5 file trong gói zip (lấy bản mới nhất mỗi loại: Beam saw bản 20.10new, UV bản (1), Ép nóng bản (1), Veneer bản 20/10) và 3 hình (thợ sơn tuần 42, cào cước 16/10, bắn cát 15/10). Chỉ lấy dòng từ 05/10 đến 20/10. UV (báo cáo ngày đến 11/10, phát sinh đến 13/10) và Ép nóng (đến 6/10) chưa có số liệu mới.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3. Tất cả giờ công trong bảng khớp với số giờ trong nguồn (sheet "Đối chiếu nguồn"). Tổng giờ công xem sheet "Đối chiếu nguồn".</t>
   </si>
   <si>
     <t xml:space="preserve">4. UV báo cáo ngày: báo cáo ghi giờ = 8 giờ x HC làm việc + 4 giờ x HC tăng ca. Tôi tách mỗi ngày thành 2 dòng (ca thường 7:30-15:30; tăng ca 15:30-19:30) để ra đúng số giờ báo cáo. Tiền lệ trong file ghi 1 dòng/ngày (7:30-19:30), cần xác nhận cách ghi.</t>
@@ -614,7 +611,7 @@
     <t xml:space="preserve">6. UV: file báo cáo ngày chỉ đến 11/10; chưa có số liệu từ 12/10. UV phát sinh 12/10 có 23 mã hàng SLAT nhưng chỉ 2 dòng có giờ (HC 1, 9:30-20:00 và 7:30-15:00); danh sách mã ở sheet "Chi tiết mã hàng". Bộ phận ghi "QC" (báo cáo ghi "QC A HIẾU"), cần xác nhận.</t>
   </si>
   <si>
-    <t xml:space="preserve">7. Beam saw: 14 dòng từ 08/10 đến 20/10. Dòng CZ567F09 ngày 20/10 ghi 18:15-18:13 (giờ kết thúc nhỏ hơn giờ bắt đầu), cần xác nhận giờ đúng (tô cam). 3 dòng ngày 19/10 (18:00-18:07) trên hệ thống đang nhập ngày 18/10, nguồn ghi ngày 19/10, cần kiểm tra lại. Khu vực ghi RC - PANEL (Raw Cutting, người dùng xác nhận 20/10). Bộ phận lấy từ cột Charge to: Machining CNC và Machining ghi "Machining"; "QA ..." ghi "QC"; 4 dòng ngày 16/10 và 20/10 là "Unassigned" (chưa phân công), cần xác định bộ phận (tô cam).</t>
+    <t xml:space="preserve">7. Beam saw: 14 dòng từ 08/10 đến 20/10.  Dòng CZ567F09 ngày 20/10 đã được sửa trong file nguồn bản 20.10new thành 18:15-18:18. 3 dòng ngày 19/10 (18:00-18:07) trên hệ thống đang nhập ngày 18/10, nguồn ghi ngày 19/10, cần kiểm tra lại. Khu vực ghi RC - PANEL (Raw Cutting, người dùng xác nhận 20/10). Bộ phận lấy từ cột Charge to: Machining CNC và Machining ghi "Machining"; "QA ..." ghi "QC"; 4 dòng ngày 16/10 và 20/10 là "Unassigned" (chưa phân công), cần xác định bộ phận (tô cam).</t>
   </si>
   <si>
     <t xml:space="preserve">8. Ép nóng: 3 nhóm (5/10 hỗ trợ P1 4 người 16 giờ; 5/10 ép lót 5 người 30 giờ; 6/10 ép chính 5 người 55 giờ). Mỗi nhóm có nhiều mã hàng cùng một ca nên ghi một dòng, mã hàng nối bằng "+" (xem sheet Chi tiết). Đừng nhân giờ cho từng mã. Giờ bắt đầu 6:30 hiếm, nên xác nhận.</t>
@@ -3681,7 +3678,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="46" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="8" t="str">
         <f aca="false">"W"&amp;WEEKNUM(B46,21)</f>
         <v>W43</v>
@@ -3713,24 +3710,24 @@
         <v>102</v>
       </c>
       <c r="L46" s="10" t="s">
-        <v>104</v>
+        <v>84</v>
       </c>
       <c r="M46" s="11" t="n">
         <v>0.760416666666667</v>
       </c>
       <c r="N46" s="11" t="n">
-        <v>0.760416666666667</v>
+        <v>0.7625</v>
       </c>
       <c r="O46" s="12" t="n">
         <f aca="false">(N46-M46)*24</f>
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="P46" s="8" t="n">
         <v>3</v>
       </c>
       <c r="Q46" s="12" t="n">
         <f aca="false">P46*O46</f>
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="R46" s="8" t="s">
         <v>41</v>
@@ -3745,7 +3742,7 @@
         <v>46315</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D47" s="3"/>
       <c r="E47" s="3" t="n">
@@ -3768,7 +3765,7 @@
         <v>60</v>
       </c>
       <c r="L47" s="5" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="M47" s="6" t="n">
         <v>0.375</v>
@@ -3800,7 +3797,7 @@
         <v>46315</v>
       </c>
       <c r="C48" s="10" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D48" s="8"/>
       <c r="E48" s="8" t="n">
@@ -3817,13 +3814,13 @@
         <v>22</v>
       </c>
       <c r="J48" s="8" t="s">
+        <v>106</v>
+      </c>
+      <c r="K48" s="10" t="s">
         <v>107</v>
       </c>
-      <c r="K48" s="10" t="s">
+      <c r="L48" s="10" t="s">
         <v>108</v>
-      </c>
-      <c r="L48" s="10" t="s">
-        <v>109</v>
       </c>
       <c r="M48" s="11" t="n">
         <v>0.416666666666667</v>
@@ -3855,7 +3852,7 @@
         <v>46315</v>
       </c>
       <c r="C49" s="5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D49" s="3"/>
       <c r="E49" s="3" t="n">
@@ -3878,7 +3875,7 @@
         <v>60</v>
       </c>
       <c r="L49" s="5" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="M49" s="6" t="n">
         <v>0.416666666666667</v>
@@ -3903,16 +3900,16 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="P50" s="18" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="Q50" s="19" t="n">
         <f aca="false">SUM(Q3:Q49)</f>
-        <v>1766.18333333333</v>
+        <v>1766.33333333333</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="20" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
   </sheetData>
@@ -3944,18 +3941,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="21" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="B3" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="C3" s="2" t="s">
         <v>115</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>116</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>26</v>
@@ -3982,7 +3979,7 @@
         <v>80</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3990,7 +3987,7 @@
         <v>46300</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C4" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A4,21)</f>
@@ -4038,7 +4035,7 @@
         <v>46301</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C5" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A5,21)</f>
@@ -4086,7 +4083,7 @@
         <v>46302</v>
       </c>
       <c r="B6" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C6" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A6,21)</f>
@@ -4134,7 +4131,7 @@
         <v>46303</v>
       </c>
       <c r="B7" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C7" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A7,21)</f>
@@ -4182,7 +4179,7 @@
         <v>46304</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C8" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A8,21)</f>
@@ -4230,7 +4227,7 @@
         <v>46305</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C9" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A9,21)</f>
@@ -4278,7 +4275,7 @@
         <v>46306</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C10" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A10,21)</f>
@@ -4326,7 +4323,7 @@
         <v>46307</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C11" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A11,21)</f>
@@ -4374,7 +4371,7 @@
         <v>46308</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C12" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A12,21)</f>
@@ -4422,7 +4419,7 @@
         <v>46309</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C13" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A13,21)</f>
@@ -4470,7 +4467,7 @@
         <v>46310</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C14" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A14,21)</f>
@@ -4518,7 +4515,7 @@
         <v>46311</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C15" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A15,21)</f>
@@ -4566,7 +4563,7 @@
         <v>46312</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C16" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A16,21)</f>
@@ -4614,7 +4611,7 @@
         <v>46314</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C17" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A17,21)</f>
@@ -4662,7 +4659,7 @@
         <v>46315</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C18" s="3" t="str">
         <f aca="false">"W"&amp;WEEKNUM(A18,21)</f>
@@ -4678,7 +4675,7 @@
       </c>
       <c r="F18" s="23" t="n">
         <f aca="false">SUMIFS('S32 5-10 đến 20-10'!$Q$3:$Q$49,'S32 5-10 đến 20-10'!$B$3:$B$49,$A18,'S32 5-10 đến 20-10'!$R$3:$R$49,F$3)</f>
-        <v>0.25</v>
+        <v>0.4</v>
       </c>
       <c r="G18" s="23" t="n">
         <f aca="false">SUMIFS('S32 5-10 đến 20-10'!$Q$3:$Q$49,'S32 5-10 đến 20-10'!$B$3:$B$49,$A18,'S32 5-10 đến 20-10'!$R$3:$R$49,G$3)</f>
@@ -4702,12 +4699,12 @@
       </c>
       <c r="L18" s="24" t="n">
         <f aca="false">SUM(D18:K18)</f>
-        <v>4.25</v>
+        <v>4.4</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="25" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B19" s="25"/>
       <c r="C19" s="25"/>
@@ -4721,7 +4718,7 @@
       </c>
       <c r="F19" s="24" t="n">
         <f aca="false">SUM(F4:F18)</f>
-        <v>2.35</v>
+        <v>2.5</v>
       </c>
       <c r="G19" s="24" t="n">
         <f aca="false">SUM(G4:G18)</f>
@@ -4745,25 +4742,25 @@
       </c>
       <c r="L19" s="24" t="n">
         <f aca="false">SUM(L4:L18)</f>
-        <v>1766.18333333333</v>
+        <v>1766.33333333333</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="2" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="26" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="B23" s="27" t="n">
         <f aca="false">SUMIFS('S32 5-10 đến 20-10'!$Q$3:$Q$49,'S32 5-10 đến 20-10'!$A$3:$A$49,A23)</f>
@@ -4772,7 +4769,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="26" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="B24" s="27" t="n">
         <f aca="false">SUMIFS('S32 5-10 đến 20-10'!$Q$3:$Q$49,'S32 5-10 đến 20-10'!$A$3:$A$49,A24)</f>
@@ -4781,11 +4778,11 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="26" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="B25" s="27" t="n">
         <f aca="false">SUMIFS('S32 5-10 đến 20-10'!$Q$3:$Q$49,'S32 5-10 đến 20-10'!$A$3:$A$49,A25)</f>
-        <v>4.6</v>
+        <v>4.75</v>
       </c>
     </row>
   </sheetData>
@@ -4822,19 +4819,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="D1" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>133</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>134</v>
       </c>
       <c r="F1" s="2" t="s">
         <v>13</v>
@@ -4843,19 +4840,19 @@
         <v>14</v>
       </c>
       <c r="H1" s="2" t="s">
+        <v>134</v>
+      </c>
+      <c r="I1" s="28" t="s">
         <v>135</v>
       </c>
-      <c r="I1" s="28" t="s">
+      <c r="J1" s="28" t="s">
         <v>136</v>
       </c>
-      <c r="J1" s="28" t="s">
+      <c r="K1" s="28" t="s">
         <v>137</v>
       </c>
-      <c r="K1" s="28" t="s">
+      <c r="L1" s="28" t="s">
         <v>138</v>
-      </c>
-      <c r="L1" s="28" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6408,7 +6405,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="36" t="n">
         <v>46315</v>
       </c>
@@ -6428,7 +6425,7 @@
         <v>0.760416666666667</v>
       </c>
       <c r="G45" s="39" t="n">
-        <v>0.760416666666667</v>
+        <v>0.7625</v>
       </c>
       <c r="H45" s="37" t="n">
         <v>3</v>
@@ -6440,7 +6437,7 @@
         <v>5</v>
       </c>
       <c r="K45" s="35" t="s">
-        <v>104</v>
+        <v>84</v>
       </c>
       <c r="L45" s="34" t="s">
         <v>41</v>
@@ -6472,13 +6469,13 @@
         <v>1</v>
       </c>
       <c r="I46" s="33" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="J46" s="34" t="n">
         <v>30</v>
       </c>
       <c r="K46" s="35" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="L46" s="34" t="s">
         <v>62</v>
@@ -6492,13 +6489,13 @@
         <v>21</v>
       </c>
       <c r="C47" s="38" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D47" s="37" t="s">
         <v>20</v>
       </c>
       <c r="E47" s="37" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F47" s="39" t="n">
         <v>0.416666666666667</v>
@@ -6510,13 +6507,13 @@
         <v>2</v>
       </c>
       <c r="I47" s="33" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="J47" s="34" t="n">
         <v>2</v>
       </c>
       <c r="K47" s="35" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="L47" s="34" t="s">
         <v>62</v>
@@ -6548,13 +6545,13 @@
         <v>1</v>
       </c>
       <c r="I48" s="33" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="J48" s="34" t="n">
         <v>30</v>
       </c>
       <c r="K48" s="35" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="L48" s="34" t="s">
         <v>62</v>
@@ -6562,7 +6559,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="20" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
   </sheetData>
@@ -6593,7 +6590,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="21" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="36" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6601,16 +6598,16 @@
         <v>18</v>
       </c>
       <c r="B3" s="2" t="s">
+        <v>141</v>
+      </c>
+      <c r="C3" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="D3" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>144</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>145</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6618,11 +6615,11 @@
         <v>41</v>
       </c>
       <c r="B4" s="45" t="n">
-        <v>2.35</v>
+        <v>2.5</v>
       </c>
       <c r="C4" s="46" t="n">
         <f aca="false">SUMIFS('S32 5-10 đến 20-10'!$Q$3:$Q$49,'S32 5-10 đến 20-10'!$R$3:$R$49,A4)</f>
-        <v>2.35</v>
+        <v>2.5</v>
       </c>
       <c r="D4" s="46" t="n">
         <f aca="false">C4-B4</f>
@@ -6775,15 +6772,15 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="47" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="B12" s="48" t="n">
         <f aca="false">SUM(B4:B11)</f>
-        <v>1766.1833</v>
+        <v>1766.3333</v>
       </c>
       <c r="C12" s="48" t="n">
         <f aca="false">SUM(C4:C11)</f>
-        <v>1766.18333333333</v>
+        <v>1766.33333333333</v>
       </c>
       <c r="D12" s="48" t="n">
         <f aca="false">SUM(D4:D11)</f>
@@ -6796,7 +6793,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="20" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
   </sheetData>
@@ -6827,19 +6824,19 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>18</v>
       </c>
       <c r="C1" s="2" t="s">
+        <v>146</v>
+      </c>
+      <c r="D1" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="E1" s="2" t="s">
         <v>148</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6850,10 +6847,10 @@
         <v>26</v>
       </c>
       <c r="C2" s="26" t="s">
+        <v>149</v>
+      </c>
+      <c r="D2" s="26" t="s">
         <v>150</v>
-      </c>
-      <c r="D2" s="26" t="s">
-        <v>151</v>
       </c>
       <c r="E2" s="26" t="n">
         <v>10</v>
@@ -6867,10 +6864,10 @@
         <v>26</v>
       </c>
       <c r="C3" s="26" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D3" s="26" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E3" s="26" t="n">
         <v>5</v>
@@ -6884,10 +6881,10 @@
         <v>26</v>
       </c>
       <c r="C4" s="26" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="D4" s="26" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E4" s="26" t="n">
         <v>10</v>
@@ -6901,10 +6898,10 @@
         <v>26</v>
       </c>
       <c r="C5" s="26" t="s">
+        <v>153</v>
+      </c>
+      <c r="D5" s="26" t="s">
         <v>154</v>
-      </c>
-      <c r="D5" s="26" t="s">
-        <v>155</v>
       </c>
       <c r="E5" s="26" t="n">
         <v>27</v>
@@ -6918,10 +6915,10 @@
         <v>26</v>
       </c>
       <c r="C6" s="26" t="s">
+        <v>155</v>
+      </c>
+      <c r="D6" s="26" t="s">
         <v>156</v>
-      </c>
-      <c r="D6" s="26" t="s">
-        <v>157</v>
       </c>
       <c r="E6" s="26" t="n">
         <v>23</v>
@@ -6935,10 +6932,10 @@
         <v>26</v>
       </c>
       <c r="C7" s="26" t="s">
+        <v>153</v>
+      </c>
+      <c r="D7" s="26" t="s">
         <v>154</v>
-      </c>
-      <c r="D7" s="26" t="s">
-        <v>155</v>
       </c>
       <c r="E7" s="26" t="n">
         <v>27</v>
@@ -6952,10 +6949,10 @@
         <v>26</v>
       </c>
       <c r="C8" s="26" t="s">
+        <v>155</v>
+      </c>
+      <c r="D8" s="26" t="s">
         <v>156</v>
-      </c>
-      <c r="D8" s="26" t="s">
-        <v>157</v>
       </c>
       <c r="E8" s="26" t="n">
         <v>23</v>
@@ -6969,10 +6966,10 @@
         <v>62</v>
       </c>
       <c r="C9" s="26" t="s">
+        <v>157</v>
+      </c>
+      <c r="D9" s="26" t="s">
         <v>158</v>
-      </c>
-      <c r="D9" s="26" t="s">
-        <v>159</v>
       </c>
       <c r="E9" s="26" t="n">
         <v>50</v>
@@ -6986,10 +6983,10 @@
         <v>62</v>
       </c>
       <c r="C10" s="26" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="D10" s="26" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E10" s="26" t="n">
         <v>100</v>
@@ -7003,10 +7000,10 @@
         <v>65</v>
       </c>
       <c r="C11" s="26" t="s">
+        <v>160</v>
+      </c>
+      <c r="D11" s="26" t="s">
         <v>161</v>
-      </c>
-      <c r="D11" s="26" t="s">
-        <v>162</v>
       </c>
       <c r="E11" s="26" t="n">
         <v>13</v>
@@ -7020,10 +7017,10 @@
         <v>65</v>
       </c>
       <c r="C12" s="26" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="D12" s="26" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E12" s="26" t="n">
         <v>13</v>
@@ -7037,10 +7034,10 @@
         <v>65</v>
       </c>
       <c r="C13" s="26" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D13" s="26" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E13" s="26" t="n">
         <v>13</v>
@@ -7054,10 +7051,10 @@
         <v>65</v>
       </c>
       <c r="C14" s="26" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="D14" s="26" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E14" s="26" t="n">
         <v>13</v>
@@ -7071,10 +7068,10 @@
         <v>65</v>
       </c>
       <c r="C15" s="26" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D15" s="26" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E15" s="26" t="n">
         <v>13</v>
@@ -7088,10 +7085,10 @@
         <v>65</v>
       </c>
       <c r="C16" s="26" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="D16" s="26" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E16" s="26" t="n">
         <v>13</v>
@@ -7105,10 +7102,10 @@
         <v>65</v>
       </c>
       <c r="C17" s="26" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="D17" s="26" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E17" s="26" t="n">
         <v>13</v>
@@ -7122,10 +7119,10 @@
         <v>65</v>
       </c>
       <c r="C18" s="26" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="D18" s="26" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E18" s="26" t="n">
         <v>13</v>
@@ -7139,10 +7136,10 @@
         <v>65</v>
       </c>
       <c r="C19" s="26" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="D19" s="26" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E19" s="26" t="n">
         <v>13</v>
@@ -7156,10 +7153,10 @@
         <v>65</v>
       </c>
       <c r="C20" s="26" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D20" s="26" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E20" s="26" t="n">
         <v>13</v>
@@ -7173,10 +7170,10 @@
         <v>65</v>
       </c>
       <c r="C21" s="26" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="D21" s="26" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E21" s="26" t="n">
         <v>13</v>
@@ -7190,10 +7187,10 @@
         <v>65</v>
       </c>
       <c r="C22" s="26" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="D22" s="26" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E22" s="26" t="n">
         <v>13</v>
@@ -7207,10 +7204,10 @@
         <v>65</v>
       </c>
       <c r="C23" s="26" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="D23" s="26" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E23" s="26" t="n">
         <v>13</v>
@@ -7224,10 +7221,10 @@
         <v>65</v>
       </c>
       <c r="C24" s="26" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="D24" s="26" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E24" s="26" t="n">
         <v>13</v>
@@ -7241,10 +7238,10 @@
         <v>65</v>
       </c>
       <c r="C25" s="26" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D25" s="26" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E25" s="26" t="n">
         <v>455</v>
@@ -7258,10 +7255,10 @@
         <v>65</v>
       </c>
       <c r="C26" s="26" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D26" s="26" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E26" s="26" t="n">
         <v>299</v>
@@ -7275,10 +7272,10 @@
         <v>65</v>
       </c>
       <c r="C27" s="26" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="D27" s="26" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E27" s="26" t="n">
         <v>286</v>
@@ -7292,10 +7289,10 @@
         <v>65</v>
       </c>
       <c r="C28" s="26" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="D28" s="26" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E28" s="26" t="n">
         <v>1092</v>
@@ -7309,10 +7306,10 @@
         <v>65</v>
       </c>
       <c r="C29" s="26" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="D29" s="26" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E29" s="26" t="n">
         <v>156</v>
@@ -7326,10 +7323,10 @@
         <v>65</v>
       </c>
       <c r="C30" s="26" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="D30" s="26" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E30" s="26" t="n">
         <v>13</v>
@@ -7343,10 +7340,10 @@
         <v>65</v>
       </c>
       <c r="C31" s="26" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="D31" s="26" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E31" s="26" t="n">
         <v>13</v>
@@ -7360,10 +7357,10 @@
         <v>65</v>
       </c>
       <c r="C32" s="26" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="D32" s="26" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E32" s="26" t="n">
         <v>13</v>
@@ -7377,10 +7374,10 @@
         <v>65</v>
       </c>
       <c r="C33" s="26" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="D33" s="26" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="E33" s="26" t="n">
         <v>13</v>
@@ -7397,7 +7394,7 @@
         <v>74</v>
       </c>
       <c r="D34" s="26" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E34" s="26" t="n">
         <v>4</v>
@@ -7411,10 +7408,10 @@
         <v>62</v>
       </c>
       <c r="C35" s="26" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D35" s="26" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="E35" s="26" t="n">
         <v>30</v>
@@ -7428,10 +7425,10 @@
         <v>62</v>
       </c>
       <c r="C36" s="26" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D36" s="26" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="E36" s="26" t="n">
         <v>2</v>
@@ -7445,10 +7442,10 @@
         <v>62</v>
       </c>
       <c r="C37" s="26" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D37" s="26" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="E37" s="26" t="n">
         <v>30</v>
@@ -7478,62 +7475,62 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="50" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="51" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="51" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="51" t="s">
         <v>189</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="51" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="51" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="51" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="51" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="51" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="51" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="37.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="51" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="51" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="25.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="51" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
     </row>
   </sheetData>

</xml_diff>